<commit_message>
Add project-type classification (QDA/QD/OTHER/NOT_A_PROJECT)
Add classify_project_type() to categorize each project by the kind of
research artefact it is, based on its recorded file types: QDA_PROJECT
(has a recognised QDA-software file), QD_PROJECT (has primary qualitative
data but no QDA file), OTHER_PROJECT (files present but none recognised as
primary data), or NOT_A_PROJECT (no files recorded at all). Store it on
CLASSIFICATIONS with a migration, and use it in the classification-table
XLSX instead of a hardcoded literal.

Also add 23123639-sq26-classification.db, the classified database named
per the SQ26 Results Data form's required convention.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/23123639_SQ26_Part2_Classification.xlsx
+++ b/23123639_SQ26_Part2_Classification.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>NOT_A_PROJECT</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>OTHER_PROJECT</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">

</xml_diff>